<commit_message>
Add data completeness summaries
</commit_message>
<xml_diff>
--- a/input/kpi_dictionary_template.example.xlsx
+++ b/input/kpi_dictionary_template.example.xlsx
@@ -1058,7 +1058,7 @@
           <t>KPI_Name_TH</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>KPI_Name_EN</t>
         </is>
@@ -1068,7 +1068,7 @@
           <t>Definition_TH</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Objective_TH</t>
         </is>
@@ -1088,12 +1088,12 @@
           <t>Denominator_Definition</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Numerator_CodeSet</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Denominator_CodeSet</t>
         </is>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">

</xml_diff>